<commit_message>
Improve accuracy of financial calculations by adjusting rounding precision
Update the `safeFormulaValue` helper in `workbook-helpers.ts` to use higher precision for rounding numerical results, ensuring financial calculations, especially percentages, are not truncated. Add `qa:parity` script to `package.json`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8a1dc927-62de-4161-963a-3067eac7a820
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/mgp02ba
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Lender_Pro_Forma_Charter_Public_Funding.xlsx
+++ b/artifacts/api-server/qa-output/Lender_Pro_Forma_Charter_Public_Funding.xlsx
@@ -1600,7 +1600,7 @@
       </c>
       <c r="G7" s="18">
         <f>Assumptions!D16*Assumptions!D22*(1+Assumptions!D23)^4</f>
-        <v>4979187.94</v>
+        <v>4979187.936</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
@@ -1621,11 +1621,11 @@
       </c>
       <c r="F8" s="18">
         <f>Assumptions!D15*Assumptions!D24*(1+Assumptions!D25)^3</f>
-        <v>122931.79</v>
+        <v>122931.7875</v>
       </c>
       <c r="G8" s="18">
         <f>Assumptions!D16*Assumptions!D24*(1+Assumptions!D25)^4</f>
-        <v>135061.06</v>
+        <v>135061.0572</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
@@ -1671,11 +1671,11 @@
       </c>
       <c r="F10" s="20">
         <f>F6+F7+F8+F9</f>
-        <v>4829391.29</v>
+        <v>4829391.2875</v>
       </c>
       <c r="G10" s="20">
         <f>G6+G7+G8+G9</f>
-        <v>5244248.99</v>
+        <v>5244248.9932</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
@@ -1717,15 +1717,15 @@
       </c>
       <c r="E13" s="18">
         <f>E12*Assumptions!D33*(1+Assumptions!D34)^2</f>
-        <v>1211203.01</v>
+        <v>1211203.0075</v>
       </c>
       <c r="F13" s="18">
         <f>F12*Assumptions!D33*(1+Assumptions!D34)^3</f>
-        <v>1596850.05</v>
+        <v>1596850.045088</v>
       </c>
       <c r="G13" s="18">
         <f>G12*Assumptions!D33*(1+Assumptions!D34)^4</f>
-        <v>1747552.77</v>
+        <v>1747552.76809318</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="G14" s="18">
         <f>Assumptions!D39*Assumptions!D40*(1+Assumptions!D41)^4</f>
-        <v>551499.32</v>
+        <v>551499.3169</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
@@ -1759,23 +1759,23 @@
       </c>
       <c r="C15" s="18">
         <f>(C13+C14)*Assumptions!D42</f>
-        <v>253497.19</v>
+        <v>253497.18888889</v>
       </c>
       <c r="D15" s="18">
         <f>(D13+D14)*Assumptions!D42</f>
-        <v>349270.37</v>
+        <v>349270.36663333</v>
       </c>
       <c r="E15" s="18">
         <f>(E13+E14)*Assumptions!D42</f>
-        <v>463535.12</v>
+        <v>463535.11756389</v>
       </c>
       <c r="F15" s="18">
         <f>(F13+F14)*Assumptions!D42</f>
-        <v>570978.88</v>
+        <v>570978.88032912</v>
       </c>
       <c r="G15" s="18">
         <f>(G13+G14)*Assumptions!D42</f>
-        <v>615635.06</v>
+        <v>615635.05831484</v>
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
@@ -1784,23 +1784,23 @@
       </c>
       <c r="C16" s="20">
         <f>C13+C14+C15</f>
-        <v>1200167.19</v>
+        <v>1200167.18888889</v>
       </c>
       <c r="D16" s="20">
         <f>D13+D14+D15</f>
-        <v>1653599.54</v>
+        <v>1653599.53663333</v>
       </c>
       <c r="E16" s="20">
         <f>E13+E14+E15</f>
-        <v>2194579.13</v>
+        <v>2194579.12506389</v>
       </c>
       <c r="F16" s="20">
         <f>F13+F14+F15</f>
-        <v>2703265.16</v>
+        <v>2703265.15541712</v>
       </c>
       <c r="G16" s="20">
         <f>G13+G14+G15</f>
-        <v>2914687.14</v>
+        <v>2914687.14330802</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
@@ -1821,11 +1821,11 @@
       </c>
       <c r="F18" s="18">
         <f>Assumptions!D46*(1+Assumptions!D47)^3</f>
-        <v>308149.01</v>
+        <v>308149.014</v>
       </c>
       <c r="G18" s="18">
         <f>Assumptions!D46*(1+Assumptions!D47)^4</f>
-        <v>317393.48</v>
+        <v>317393.48442</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
@@ -1863,19 +1863,19 @@
       </c>
       <c r="D20" s="18">
         <f>Assumptions!D13*Assumptions!D50*(1+Assumptions!D51)^1</f>
-        <v>240333.33</v>
+        <v>240333.33333333</v>
       </c>
       <c r="E20" s="18">
         <f>Assumptions!D14*Assumptions!D50*(1+Assumptions!D51)^2</f>
-        <v>618858.33</v>
+        <v>618858.33333333</v>
       </c>
       <c r="F20" s="18">
         <f>Assumptions!D15*Assumptions!D50*(1+Assumptions!D51)^3</f>
-        <v>1327966.84</v>
+        <v>1327966.84027778</v>
       </c>
       <c r="G20" s="18">
         <f>Assumptions!D16*Assumptions!D50*(1+Assumptions!D51)^4</f>
-        <v>2431654.84</v>
+        <v>2431654.83641975</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
@@ -1892,15 +1892,15 @@
       </c>
       <c r="E21" s="18">
         <f>Assumptions!D52*(1+Assumptions!D53)^2</f>
-        <v>713160.56</v>
+        <v>713160.55555556</v>
       </c>
       <c r="F21" s="18">
         <f>Assumptions!D52*(1+Assumptions!D53)^3</f>
-        <v>1122237.37</v>
+        <v>1122237.3742284</v>
       </c>
       <c r="G21" s="18">
         <f>Assumptions!D52*(1+Assumptions!D53)^4</f>
-        <v>1765965.2</v>
+        <v>1765965.20138996</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
@@ -1913,19 +1913,19 @@
       </c>
       <c r="D22" s="20">
         <f>D18+D19+D20+D21</f>
-        <v>983993.33</v>
+        <v>983993.33333333</v>
       </c>
       <c r="E22" s="20">
         <f>E18+E19+E20+E21</f>
-        <v>1631192.69</v>
+        <v>1631192.68888889</v>
       </c>
       <c r="F22" s="20">
         <f>F18+F19+F20+F21</f>
-        <v>2758353.23</v>
+        <v>2758353.22850617</v>
       </c>
       <c r="G22" s="20">
         <f>G18+G19+G20+G21</f>
-        <v>4515013.52</v>
+        <v>4515013.52222971</v>
       </c>
     </row>
   </sheetData>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="G7" s="18">
         <f>Drivers!G7</f>
-        <v>4979187.94</v>
+        <v>4979187.936</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
@@ -2075,11 +2075,11 @@
       </c>
       <c r="F8" s="18">
         <f>Drivers!F8</f>
-        <v>122931.79</v>
+        <v>122931.7875</v>
       </c>
       <c r="G8" s="18">
         <f>Drivers!G8</f>
-        <v>135061.06</v>
+        <v>135061.0572</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
@@ -2125,11 +2125,11 @@
       </c>
       <c r="F10" s="20">
         <f>Drivers!F10</f>
-        <v>4829391.29</v>
+        <v>4829391.2875</v>
       </c>
       <c r="G10" s="20">
         <f>Drivers!G10</f>
-        <v>5244248.99</v>
+        <v>5244248.9932</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
@@ -2138,23 +2138,23 @@
       </c>
       <c r="C12" s="18">
         <f>Drivers!C16</f>
-        <v>1200167.19</v>
+        <v>1200167.18888889</v>
       </c>
       <c r="D12" s="18">
         <f>Drivers!D16</f>
-        <v>1653599.54</v>
+        <v>1653599.53663333</v>
       </c>
       <c r="E12" s="18">
         <f>Drivers!E16</f>
-        <v>2194579.13</v>
+        <v>2194579.12506389</v>
       </c>
       <c r="F12" s="18">
         <f>Drivers!F16</f>
-        <v>2703265.16</v>
+        <v>2703265.15541712</v>
       </c>
       <c r="G12" s="18">
         <f>Drivers!G16</f>
-        <v>2914687.14</v>
+        <v>2914687.14330802</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
@@ -2167,19 +2167,19 @@
       </c>
       <c r="D13" s="18">
         <f>Drivers!D22</f>
-        <v>983993.33</v>
+        <v>983993.33333333</v>
       </c>
       <c r="E13" s="18">
         <f>Drivers!E22</f>
-        <v>1631192.69</v>
+        <v>1631192.68888889</v>
       </c>
       <c r="F13" s="18">
         <f>Drivers!F22</f>
-        <v>2758353.23</v>
+        <v>2758353.22850617</v>
       </c>
       <c r="G13" s="18">
         <f>Drivers!G22</f>
-        <v>4515013.52</v>
+        <v>4515013.52222971</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
@@ -2188,23 +2188,23 @@
       </c>
       <c r="C15" s="20">
         <f>C12+C13</f>
-        <v>1854167.19</v>
+        <v>1854167.18888889</v>
       </c>
       <c r="D15" s="20">
         <f>D12+D13</f>
-        <v>2637592.87</v>
+        <v>2637592.86996667</v>
       </c>
       <c r="E15" s="20">
         <f>E12+E13</f>
-        <v>3825771.81</v>
+        <v>3825771.81395278</v>
       </c>
       <c r="F15" s="20">
         <f>F12+F13</f>
-        <v>5461618.38</v>
+        <v>5461618.38392329</v>
       </c>
       <c r="G15" s="20">
         <f>G12+G13</f>
-        <v>7429700.67</v>
+        <v>7429700.66553774</v>
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
@@ -2213,23 +2213,23 @@
       </c>
       <c r="C16" s="21">
         <f>C10-C15</f>
-        <v>-308167.19</v>
+        <v>-308167.18888889</v>
       </c>
       <c r="D16" s="21">
         <f>D10-D15</f>
-        <v>-99792.87</v>
+        <v>-99792.86996667</v>
       </c>
       <c r="E16" s="21">
         <f>E10-E15</f>
-        <v>-10910.81</v>
+        <v>-10910.81395278</v>
       </c>
       <c r="F16" s="21">
         <f>F10-F15</f>
-        <v>-632227.1</v>
+        <v>-632227.09642329</v>
       </c>
       <c r="G16" s="21">
         <f>G10-G15</f>
-        <v>-2185451.67</v>
+        <v>-2185451.67233774</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
@@ -2238,23 +2238,23 @@
       </c>
       <c r="C17" s="22">
         <f>IF(C10&gt;0,C16/C10,0)</f>
-        <v>-0.2</v>
+        <v>-0.19933195</v>
       </c>
       <c r="D17" s="22">
         <f>IF(D10&gt;0,D16/D10,0)</f>
-        <v>-0.04</v>
-      </c>
-      <c r="E17" s="22" t="str">
+        <v>-0.03932259</v>
+      </c>
+      <c r="E17" s="22">
         <f>IF(E10&gt;0,E16/E10,0)</f>
-        <v>0</v>
+        <v>-0.00286008</v>
       </c>
       <c r="F17" s="22">
         <f>IF(F10&gt;0,F16/F10,0)</f>
-        <v>-0.13</v>
+        <v>-0.13091238</v>
       </c>
       <c r="G17" s="22">
         <f>IF(G10&gt;0,G16/G10,0)</f>
-        <v>-0.42</v>
+        <v>-0.41673301</v>
       </c>
     </row>
   </sheetData>
@@ -2317,23 +2317,23 @@
       </c>
       <c r="C4" s="18">
         <f>'5-Year P&amp;L'!C16</f>
-        <v>-308167.19</v>
+        <v>-308167.18888889</v>
       </c>
       <c r="D4" s="18">
         <f>'5-Year P&amp;L'!D16</f>
-        <v>-99792.87</v>
+        <v>-99792.86996667</v>
       </c>
       <c r="E4" s="18">
         <f>'5-Year P&amp;L'!E16</f>
-        <v>-10910.81</v>
+        <v>-10910.81395278</v>
       </c>
       <c r="F4" s="18">
         <f>'5-Year P&amp;L'!F16</f>
-        <v>-632227.1</v>
+        <v>-632227.09642329</v>
       </c>
       <c r="G4" s="18">
         <f>'5-Year P&amp;L'!G16</f>
-        <v>-2185451.67</v>
+        <v>-2185451.67233774</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
@@ -2367,23 +2367,23 @@
       </c>
       <c r="C7" s="18">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
-        <v>49824.61</v>
+        <v>49824.60522118</v>
       </c>
       <c r="D7" s="18">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
-        <v>49824.61</v>
+        <v>49824.60522118</v>
       </c>
       <c r="E7" s="18">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
-        <v>49824.61</v>
+        <v>49824.60522118</v>
       </c>
       <c r="F7" s="18">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
-        <v>49824.61</v>
+        <v>49824.60522118</v>
       </c>
       <c r="G7" s="18">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
-        <v>49824.61</v>
+        <v>49824.60522118</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
@@ -2392,23 +2392,23 @@
       </c>
       <c r="C8" s="20">
         <f>C6+C7</f>
-        <v>164824.61</v>
+        <v>164824.60522118</v>
       </c>
       <c r="D8" s="20">
         <f>D6+D7</f>
-        <v>164824.61</v>
+        <v>164824.60522118</v>
       </c>
       <c r="E8" s="20">
         <f>E6+E7</f>
-        <v>164824.61</v>
+        <v>164824.60522118</v>
       </c>
       <c r="F8" s="20">
         <f>F6+F7</f>
-        <v>164824.61</v>
+        <v>164824.60522118</v>
       </c>
       <c r="G8" s="20">
         <f>G6+G7</f>
-        <v>164824.61</v>
+        <v>164824.60522118</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
@@ -2417,23 +2417,23 @@
       </c>
       <c r="C10" s="23">
         <f>IF(C8&gt;0,C4/C8,IF(C4&gt;0,99.9,0))</f>
-        <v>-1.87</v>
+        <v>-1.86966739</v>
       </c>
       <c r="D10" s="23">
         <f>IF(D8&gt;0,D4/D8,IF(D4&gt;0,99.9,0))</f>
-        <v>-0.61</v>
+        <v>-0.60544886</v>
       </c>
       <c r="E10" s="23">
         <f>IF(E8&gt;0,E4/E8,IF(E4&gt;0,99.9,0))</f>
-        <v>-0.07</v>
+        <v>-0.06619651</v>
       </c>
       <c r="F10" s="23">
         <f>IF(F8&gt;0,F4/F8,IF(F4&gt;0,99.9,0))</f>
-        <v>-3.84</v>
+        <v>-3.83575678</v>
       </c>
       <c r="G10" s="23">
         <f>IF(G8&gt;0,G4/G8,IF(G4&gt;0,99.9,0))</f>
-        <v>-13.26</v>
+        <v>-13.25925622</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
@@ -2442,23 +2442,23 @@
       </c>
       <c r="C12" s="18">
         <f>C4-C8</f>
-        <v>-472991.79</v>
+        <v>-472991.79411007</v>
       </c>
       <c r="D12" s="18">
         <f>D4-D8</f>
-        <v>-264617.48</v>
+        <v>-264617.47518785</v>
       </c>
       <c r="E12" s="18">
         <f>E4-E8</f>
-        <v>-175735.42</v>
+        <v>-175735.41917396</v>
       </c>
       <c r="F12" s="18">
         <f>F4-F8</f>
-        <v>-797051.7</v>
+        <v>-797051.70164447</v>
       </c>
       <c r="G12" s="18">
         <f>G4-G8</f>
-        <v>-2350276.28</v>
+        <v>-2350276.27755892</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
@@ -2467,23 +2467,23 @@
       </c>
       <c r="C14" s="24">
         <f>Assumptions!D57+C12</f>
-        <v>-472991.79</v>
+        <v>-472991.79411007</v>
       </c>
       <c r="D14" s="24">
         <f>C14+D12</f>
-        <v>-737609.27</v>
+        <v>-737609.26929791</v>
       </c>
       <c r="E14" s="24">
         <f>D14+E12</f>
-        <v>-913344.69</v>
+        <v>-913344.68847187</v>
       </c>
       <c r="F14" s="24">
         <f>E14+F12</f>
-        <v>-1710396.39</v>
+        <v>-1710396.39011634</v>
       </c>
       <c r="G14" s="24">
         <f>F14+G12</f>
-        <v>-4060672.67</v>
+        <v>-4060672.66767526</v>
       </c>
     </row>
   </sheetData>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="C4" s="22">
         <f>Assumptions!D60</f>
-        <v>0.06</v>
+        <v>0.0575</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="C6" s="26">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
-        <v>49824.61</v>
+        <v>49824.60522118</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="C8" s="23">
         <f>'Cash Flow &amp; DSCR'!C10</f>
-        <v>-1.87</v>
+        <v>-1.86966739</v>
       </c>
     </row>
   </sheetData>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="C9" s="18">
         <f>Drivers!G10</f>
-        <v>5244248.99</v>
+        <v>5244248.9932</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="C10" s="24">
         <f>'5-Year P&amp;L'!G16</f>
-        <v>-2185451.67</v>
+        <v>-2185451.67233774</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">

</xml_diff>